<commit_message>
Use e for English language code; empty still defaults to English
</commit_message>
<xml_diff>
--- a/templates/WPS库存协作模板.xlsx
+++ b/templates/WPS库存协作模板.xlsx
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="72" customWidth="1" min="1" max="1"/>
@@ -575,38 +575,35 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr"/>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>系列  编号  语言  闪  数量  备注</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>系列  编号  语言  闪  数量  备注</t>
+          <t>语言：e=英文  z=中文  j=日文  o=其他（空默认 e）</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>语言：空=英文  z=中文  j=日文  o=其他（只支持这些）</t>
+          <t>闪：空或0=非闪  1=闪</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>闪：空或0=非闪  1=闪</t>
+          <t>数量：空=1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>数量：空=1</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>卖光：删行。同卡合并一行改数量。</t>
         </is>
@@ -645,7 +642,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>语言：空=英  z=中  j=日  o=其他 ｜ 闪：空/0=否  1=是 ｜ 数量：空=1 ｜ 卖光删行</t>
+          <t>语言：e=英 z=中 j=日 o=其他（空默认e）｜闪：空/0=否 1=是｜数量：空=1｜卖光删行</t>
         </is>
       </c>
     </row>
@@ -676,7 +673,7 @@
       <c r="B6" s="6" t="inlineStr"/>
       <c r="C6" s="7" t="n"/>
     </row>
-    <row r="8" ht="20" customHeight="1">
+    <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>系列</t>
@@ -747,7 +744,11 @@
           <t>224</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr"/>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>e</t>
+        </is>
+      </c>
       <c r="D10" s="9" t="n">
         <v>0</v>
       </c>
@@ -1498,7 +1499,7 @@
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="C9:C200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"z,j,o"</formula1>
+      <formula1>"e,z,j,o"</formula1>
     </dataValidation>
     <dataValidation sqref="D9:D200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"0,1"</formula1>
@@ -1536,7 +1537,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>语言：空=英  z=中  j=日  o=其他 ｜ 闪：空/0=否  1=是 ｜ 数量：空=1 ｜ 卖光删行</t>
+          <t>语言：e=英 z=中 j=日 o=其他（空默认e）｜闪：空/0=否 1=是｜数量：空=1｜卖光删行</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1580,7 @@
       </c>
       <c r="C6" s="7" t="n"/>
     </row>
-    <row r="8" ht="20" customHeight="1">
+    <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>系列</t>
@@ -1646,9 +1647,17 @@
           <t>224</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr"/>
-      <c r="D10" s="9" t="inlineStr"/>
-      <c r="E10" s="9" t="inlineStr"/>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>e</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="F10" s="9" t="inlineStr"/>
     </row>
     <row r="11">
@@ -1662,13 +1671,13 @@
           <t>185</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr"/>
-      <c r="D11" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="9" t="n">
-        <v>1</v>
-      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>e</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr"/>
+      <c r="E11" s="9" t="inlineStr"/>
       <c r="F11" s="9" t="inlineStr"/>
     </row>
     <row r="12">
@@ -2409,7 +2418,7 @@
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="C9:C200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"z,j,o"</formula1>
+      <formula1>"e,z,j,o"</formula1>
     </dataValidation>
     <dataValidation sqref="D9:D200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"0,1"</formula1>

</xml_diff>

<commit_message>
Update WPS xlsx help sheets with copy-sheet and QQ instructions
</commit_message>
<xml_diff>
--- a/templates/WPS库存协作模板.xlsx
+++ b/templates/WPS库存协作模板.xlsx
@@ -534,16 +534,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="72" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>WPS 库存表 · 简规</t>
+          <t>WPS 库存 · 怎么用</t>
         </is>
       </c>
     </row>
@@ -553,59 +553,76 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>管理员：复制「模板」→ 改名给每个卖家 → 开编辑权限。</t>
+          <t>1. 打开云文档（链接由群主分享）</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>卖家：只改自己的表。每天统一上网站。</t>
+          <t>2. 找到名为「模板」的工作表</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>3. 在「模板」上【右键】→【创建副本】</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>昵称 / 城市 / 联系：表上方三格。</t>
+          <t>4. 把副本【重命名】成你自己的名字（如 claystan）</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>系列  编号  语言  闪  数量  备注</t>
+          <t>5. 只改自己的表：上方填昵称/城市/联系，下方填卡牌</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>语言：e=英文  z=中文  j=日文  o=其他（空默认 e）</t>
+          <t>6. 若没有编辑权限 / 无法创建副本：联系 QQ 417592443 申请</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>闪：空或0=非闪  1=闪</t>
-        </is>
-      </c>
+      <c r="A10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>数量：空=1</t>
+          <t>语言：e=英 z=中 j=日 o=其他（空=e）</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>卖光：删行。同卡合并一行改数量。</t>
+          <t>闪：空/0=否  1=是   数量：空=1   卖光：删行</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>保存后等每天统一更新网站即可。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>文档：https://www.kdocs.cn/l/cgyl3WizNfp7</t>
         </is>
       </c>
     </row>
@@ -639,10 +656,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1">
+    <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>语言：e=英 z=中 j=日 o=其他（空默认e）｜闪：空/0=否 1=是｜数量：空=1｜卖光删行</t>
+          <t>语言 e/z/j/o（空=e）｜闪 0/1（空=0）｜数量空=1｜卖光删行｜无权限 QQ 417592443</t>
         </is>
       </c>
     </row>
@@ -756,26 +773,12 @@
       <c r="F10" s="9" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>iko</t>
-        </is>
-      </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>185</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>j</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="inlineStr"/>
-      <c r="E11" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" s="9" t="inlineStr"/>
+      <c r="A11" s="10" t="inlineStr"/>
+      <c r="B11" s="10" t="inlineStr"/>
+      <c r="C11" s="10" t="inlineStr"/>
+      <c r="D11" s="10" t="inlineStr"/>
+      <c r="E11" s="10" t="inlineStr"/>
+      <c r="F11" s="10" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr"/>
@@ -1534,10 +1537,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1">
+    <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>语言：e=英 z=中 j=日 o=其他（空默认e）｜闪：空/0=否 1=是｜数量：空=1｜卖光删行</t>
+          <t>语言 e/z/j/o（空=e）｜闪 0/1（空=0）｜数量空=1｜卖光删行｜无权限 QQ 417592443</t>
         </is>
       </c>
     </row>
@@ -1661,48 +1664,20 @@
       <c r="F10" s="9" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>iko</t>
-        </is>
-      </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>185</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>e</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="inlineStr"/>
-      <c r="E11" s="9" t="inlineStr"/>
-      <c r="F11" s="9" t="inlineStr"/>
+      <c r="A11" s="10" t="inlineStr"/>
+      <c r="B11" s="10" t="inlineStr"/>
+      <c r="C11" s="10" t="inlineStr"/>
+      <c r="D11" s="10" t="inlineStr"/>
+      <c r="E11" s="10" t="inlineStr"/>
+      <c r="F11" s="10" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>rna</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>245</t>
-        </is>
-      </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>z</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" s="9" t="inlineStr"/>
+      <c r="A12" s="10" t="inlineStr"/>
+      <c r="B12" s="10" t="inlineStr"/>
+      <c r="C12" s="10" t="inlineStr"/>
+      <c r="D12" s="10" t="inlineStr"/>
+      <c r="E12" s="10" t="inlineStr"/>
+      <c r="F12" s="10" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr"/>

</xml_diff>

<commit_message>
Shorten WPS template help: drop open-doc and URL lines
</commit_message>
<xml_diff>
--- a/templates/WPS库存协作模板.xlsx
+++ b/templates/WPS库存协作模板.xlsx
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="78" customWidth="1" min="1" max="1"/>
@@ -553,76 +553,52 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>1. 打开云文档（链接由群主分享）</t>
+          <t>1. 在「模板」上【右键】→【创建副本】</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2. 找到名为「模板」的工作表</t>
+          <t>2. 把副本【重命名】成你自己的名字（如 claystan）</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>3. 在「模板」上【右键】→【创建副本】</t>
+          <t>3. 只改自己的表：上方填昵称/城市/联系，下方填卡牌</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>4. 把副本【重命名】成你自己的名字（如 claystan）</t>
+          <t>4. 若没有编辑权限 / 无法创建副本：联系 QQ 417592443 申请</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>5. 只改自己的表：上方填昵称/城市/联系，下方填卡牌</t>
-        </is>
-      </c>
+      <c r="A8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>6. 若没有编辑权限 / 无法创建副本：联系 QQ 417592443 申请</t>
+          <t>语言：e=英 z=中 j=日 o=其他（空=e）</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr"/>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>闪：空/0=否  1=是   数量：空=1   卖光：删行</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>语言：e=英 z=中 j=日 o=其他（空=e）</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>闪：空/0=否  1=是   数量：空=1   卖光：删行</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
           <t>保存后等每天统一更新网站即可。</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>文档：https://www.kdocs.cn/l/cgyl3WizNfp7</t>
         </is>
       </c>
     </row>

</xml_diff>